<commit_message>
Updated with Fixed Metrics
</commit_message>
<xml_diff>
--- a/species_prevalence.xlsx
+++ b/species_prevalence.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="106">
   <si>
     <t>Species</t>
   </si>
@@ -139,9 +139,6 @@
     <t>Giraffa camelopardalis</t>
   </si>
   <si>
-    <t>Gonocephalus chamaeleontinus</t>
-  </si>
-  <si>
     <t>Gopherus agassizii</t>
   </si>
   <si>
@@ -205,9 +202,6 @@
     <t>Morelia viridis</t>
   </si>
   <si>
-    <t>Mus musculus</t>
-  </si>
-  <si>
     <t>Mustela nigripes</t>
   </si>
   <si>
@@ -244,18 +238,12 @@
     <t>Oxyura jamaicensis</t>
   </si>
   <si>
-    <t>Pan troglodytes</t>
-  </si>
-  <si>
     <t>Panthera leo</t>
   </si>
   <si>
     <t>Panthera onca</t>
   </si>
   <si>
-    <t>Panthera pardus</t>
-  </si>
-  <si>
     <t>Panthera tigris</t>
   </si>
   <si>
@@ -341,9 +329,6 @@
   </si>
   <si>
     <t>Varecia variegata</t>
-  </si>
-  <si>
-    <t>Vicugna pacos</t>
   </si>
   <si>
     <t>Zalophus californianus</t>
@@ -689,7 +674,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G101"/>
+  <dimension ref="A1:G96"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7" s="1" customFormat="1">
@@ -723,19 +708,19 @@
         <v>8</v>
       </c>
       <c r="C2">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D2">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F2">
-        <v>0.4848484848484849</v>
+        <v>0.4516129032258064</v>
       </c>
       <c r="G2">
-        <v>0.1515151515151515</v>
+        <v>0.09677419354838709</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -815,19 +800,19 @@
         <v>8</v>
       </c>
       <c r="C6">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="D6">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="E6">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F6">
-        <v>0.5934959349593496</v>
+        <v>0.576271186440678</v>
       </c>
       <c r="G6">
-        <v>0.4390243902439024</v>
+        <v>0.4406779661016949</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -861,19 +846,19 @@
         <v>14</v>
       </c>
       <c r="C8">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D8">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E8">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F8">
-        <v>0.40625</v>
+        <v>0.3870967741935484</v>
       </c>
       <c r="G8">
-        <v>0.28125</v>
+        <v>0.2580645161290323</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -884,19 +869,19 @@
         <v>8</v>
       </c>
       <c r="C9">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D9">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E9">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F9">
-        <v>0.5789473684210527</v>
+        <v>0.5294117647058824</v>
       </c>
       <c r="G9">
-        <v>0.4473684210526316</v>
+        <v>0.4411764705882353</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -1206,19 +1191,19 @@
         <v>8</v>
       </c>
       <c r="C23">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D23">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E23">
         <v>13</v>
       </c>
       <c r="F23">
-        <v>0.5084745762711864</v>
+        <v>0.4821428571428572</v>
       </c>
       <c r="G23">
-        <v>0.2203389830508475</v>
+        <v>0.2321428571428572</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -1390,19 +1375,19 @@
         <v>30</v>
       </c>
       <c r="C31">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="D31">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="E31">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="F31">
-        <v>0.477124183006536</v>
+        <v>0.4557823129251701</v>
       </c>
       <c r="G31">
-        <v>0.3725490196078431</v>
+        <v>0.3469387755102041</v>
       </c>
     </row>
     <row r="32" spans="1:7">
@@ -1436,19 +1421,19 @@
         <v>14</v>
       </c>
       <c r="C33">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D33">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="E33">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F33">
-        <v>0.5238095238095238</v>
+        <v>0.05</v>
       </c>
       <c r="G33">
-        <v>0.1904761904761905</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="34" spans="1:7">
@@ -1456,22 +1441,22 @@
         <v>42</v>
       </c>
       <c r="B34" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="C34">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="D34">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E34">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F34">
-        <v>0.05</v>
+        <v>0.303030303030303</v>
       </c>
       <c r="G34">
-        <v>0.05</v>
+        <v>0.1515151515151515</v>
       </c>
     </row>
     <row r="35" spans="1:7">
@@ -1479,22 +1464,22 @@
         <v>43</v>
       </c>
       <c r="B35" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C35">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="D35">
         <v>10</v>
       </c>
       <c r="E35">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F35">
-        <v>0.303030303030303</v>
+        <v>0.3846153846153846</v>
       </c>
       <c r="G35">
-        <v>0.1515151515151515</v>
+        <v>0.3846153846153846</v>
       </c>
     </row>
     <row r="36" spans="1:7">
@@ -1502,22 +1487,22 @@
         <v>44</v>
       </c>
       <c r="B36" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="C36">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D36">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E36">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F36">
-        <v>0.3846153846153846</v>
+        <v>0.1304347826086956</v>
       </c>
       <c r="G36">
-        <v>0.3846153846153846</v>
+        <v>0.04347826086956522</v>
       </c>
     </row>
     <row r="37" spans="1:7">
@@ -1528,19 +1513,19 @@
         <v>8</v>
       </c>
       <c r="C37">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="D37">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E37">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F37">
-        <v>0.1304347826086956</v>
+        <v>0.2647058823529412</v>
       </c>
       <c r="G37">
-        <v>0.04347826086956522</v>
+        <v>0.2058823529411765</v>
       </c>
     </row>
     <row r="38" spans="1:7">
@@ -1551,19 +1536,19 @@
         <v>8</v>
       </c>
       <c r="C38">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="D38">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E38">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F38">
-        <v>0.3421052631578947</v>
+        <v>0.44</v>
       </c>
       <c r="G38">
-        <v>0.2368421052631579</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="39" spans="1:7">
@@ -1571,22 +1556,22 @@
         <v>47</v>
       </c>
       <c r="B39" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C39">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="D39">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E39">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="F39">
-        <v>0.4814814814814815</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="G39">
-        <v>0.1851851851851852</v>
+        <v>0.5714285714285714</v>
       </c>
     </row>
     <row r="40" spans="1:7">
@@ -1597,19 +1582,19 @@
         <v>14</v>
       </c>
       <c r="C40">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="D40">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E40">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F40">
-        <v>0.6666666666666666</v>
+        <v>0.5</v>
       </c>
       <c r="G40">
-        <v>0.5714285714285714</v>
+        <v>0.3823529411764706</v>
       </c>
     </row>
     <row r="41" spans="1:7">
@@ -1617,22 +1602,22 @@
         <v>49</v>
       </c>
       <c r="B41" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="C41">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="D41">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="E41">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="F41">
-        <v>0.5</v>
+        <v>0.03703703703703703</v>
       </c>
       <c r="G41">
-        <v>0.3823529411764706</v>
+        <v>0.03703703703703703</v>
       </c>
     </row>
     <row r="42" spans="1:7">
@@ -1640,22 +1625,22 @@
         <v>50</v>
       </c>
       <c r="B42" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="C42">
-        <v>27</v>
+        <v>72</v>
       </c>
       <c r="D42">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="E42">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="F42">
-        <v>0.03703703703703703</v>
+        <v>0.4583333333333333</v>
       </c>
       <c r="G42">
-        <v>0.03703703703703703</v>
+        <v>0.3055555555555556</v>
       </c>
     </row>
     <row r="43" spans="1:7">
@@ -1666,19 +1651,19 @@
         <v>8</v>
       </c>
       <c r="C43">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="D43">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="E43">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="F43">
-        <v>0.4583333333333333</v>
+        <v>0.3432835820895522</v>
       </c>
       <c r="G43">
-        <v>0.3055555555555556</v>
+        <v>0.1492537313432836</v>
       </c>
     </row>
     <row r="44" spans="1:7">
@@ -1686,22 +1671,22 @@
         <v>52</v>
       </c>
       <c r="B44" t="s">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="C44">
-        <v>67</v>
+        <v>32</v>
       </c>
       <c r="D44">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="E44">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="F44">
-        <v>0.3432835820895522</v>
+        <v>0.15625</v>
       </c>
       <c r="G44">
-        <v>0.1492537313432836</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="45" spans="1:7">
@@ -1709,22 +1694,22 @@
         <v>53</v>
       </c>
       <c r="B45" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="C45">
-        <v>32</v>
+        <v>49</v>
       </c>
       <c r="D45">
         <v>5</v>
       </c>
       <c r="E45">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F45">
-        <v>0.15625</v>
+        <v>0.1020408163265306</v>
       </c>
       <c r="G45">
-        <v>0.125</v>
+        <v>0.04081632653061224</v>
       </c>
     </row>
     <row r="46" spans="1:7">
@@ -1735,19 +1720,19 @@
         <v>8</v>
       </c>
       <c r="C46">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="D46">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E46">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="F46">
-        <v>0.1020408163265306</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="G46">
-        <v>0.04081632653061224</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="47" spans="1:7">
@@ -1758,19 +1743,19 @@
         <v>8</v>
       </c>
       <c r="C47">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="D47">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="E47">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="F47">
-        <v>0.4166666666666667</v>
+        <v>0.6</v>
       </c>
       <c r="G47">
-        <v>0.25</v>
+        <v>0.4222222222222222</v>
       </c>
     </row>
     <row r="48" spans="1:7">
@@ -1781,19 +1766,19 @@
         <v>8</v>
       </c>
       <c r="C48">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="D48">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="E48">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="F48">
-        <v>0.6</v>
+        <v>0.07407407407407407</v>
       </c>
       <c r="G48">
-        <v>0.4222222222222222</v>
+        <v>0.07407407407407407</v>
       </c>
     </row>
     <row r="49" spans="1:7">
@@ -1804,19 +1789,19 @@
         <v>8</v>
       </c>
       <c r="C49">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D49">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="E49">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F49">
-        <v>0.07407407407407407</v>
+        <v>0.3214285714285715</v>
       </c>
       <c r="G49">
-        <v>0.07407407407407407</v>
+        <v>0.1785714285714286</v>
       </c>
     </row>
     <row r="50" spans="1:7">
@@ -1824,22 +1809,22 @@
         <v>58</v>
       </c>
       <c r="B50" t="s">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="C50">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="D50">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E50">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F50">
-        <v>0.3214285714285715</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="G50">
-        <v>0.1785714285714286</v>
+        <v>0.1363636363636364</v>
       </c>
     </row>
     <row r="51" spans="1:7">
@@ -1850,19 +1835,19 @@
         <v>30</v>
       </c>
       <c r="C51">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="D51">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E51">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F51">
-        <v>0.1818181818181818</v>
+        <v>0.2</v>
       </c>
       <c r="G51">
-        <v>0.1363636363636364</v>
+        <v>0.1714285714285714</v>
       </c>
     </row>
     <row r="52" spans="1:7">
@@ -1873,19 +1858,19 @@
         <v>30</v>
       </c>
       <c r="C52">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="D52">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="E52">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="F52">
-        <v>0.2</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="G52">
-        <v>0.1714285714285714</v>
+        <v>0.2916666666666667</v>
       </c>
     </row>
     <row r="53" spans="1:7">
@@ -1893,22 +1878,22 @@
         <v>61</v>
       </c>
       <c r="B53" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="C53">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="D53">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="E53">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="F53">
-        <v>0.4285714285714285</v>
+        <v>0.09375</v>
       </c>
       <c r="G53">
-        <v>0.3061224489795918</v>
+        <v>0.0625</v>
       </c>
     </row>
     <row r="54" spans="1:7">
@@ -1916,22 +1901,22 @@
         <v>62</v>
       </c>
       <c r="B54" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="C54">
-        <v>32</v>
+        <v>78</v>
       </c>
       <c r="D54">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="E54">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F54">
-        <v>0.09375</v>
+        <v>0.2692307692307692</v>
       </c>
       <c r="G54">
-        <v>0.0625</v>
+        <v>0.1282051282051282</v>
       </c>
     </row>
     <row r="55" spans="1:7">
@@ -1942,19 +1927,19 @@
         <v>8</v>
       </c>
       <c r="C55">
-        <v>26</v>
+        <v>81</v>
       </c>
       <c r="D55">
-        <v>20</v>
+        <v>64</v>
       </c>
       <c r="E55">
-        <v>12</v>
+        <v>43</v>
       </c>
       <c r="F55">
-        <v>0.7692307692307693</v>
+        <v>0.7901234567901234</v>
       </c>
       <c r="G55">
-        <v>0.4615384615384616</v>
+        <v>0.5308641975308642</v>
       </c>
     </row>
     <row r="56" spans="1:7">
@@ -1965,19 +1950,19 @@
         <v>8</v>
       </c>
       <c r="C56">
-        <v>78</v>
+        <v>45</v>
       </c>
       <c r="D56">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="E56">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="F56">
-        <v>0.2692307692307692</v>
+        <v>0.1777777777777778</v>
       </c>
       <c r="G56">
-        <v>0.1282051282051282</v>
+        <v>0.06666666666666667</v>
       </c>
     </row>
     <row r="57" spans="1:7">
@@ -1985,22 +1970,22 @@
         <v>65</v>
       </c>
       <c r="B57" t="s">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="C57">
-        <v>95</v>
+        <v>23</v>
       </c>
       <c r="D57">
-        <v>78</v>
+        <v>2</v>
       </c>
       <c r="E57">
-        <v>51</v>
+        <v>1</v>
       </c>
       <c r="F57">
-        <v>0.8210526315789474</v>
+        <v>0.08695652173913043</v>
       </c>
       <c r="G57">
-        <v>0.5368421052631579</v>
+        <v>0.04347826086956522</v>
       </c>
     </row>
     <row r="58" spans="1:7">
@@ -2011,19 +1996,19 @@
         <v>8</v>
       </c>
       <c r="C58">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="D58">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E58">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F58">
-        <v>0.1777777777777778</v>
+        <v>0.04878048780487805</v>
       </c>
       <c r="G58">
-        <v>0.06666666666666667</v>
+        <v>0.04878048780487805</v>
       </c>
     </row>
     <row r="59" spans="1:7">
@@ -2034,19 +2019,19 @@
         <v>30</v>
       </c>
       <c r="C59">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D59">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E59">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F59">
-        <v>0.08695652173913043</v>
+        <v>0.3</v>
       </c>
       <c r="G59">
-        <v>0.04347826086956522</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="60" spans="1:7">
@@ -2057,19 +2042,19 @@
         <v>8</v>
       </c>
       <c r="C60">
-        <v>41</v>
+        <v>96</v>
       </c>
       <c r="D60">
-        <v>2</v>
+        <v>36</v>
       </c>
       <c r="E60">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="F60">
-        <v>0.04878048780487805</v>
+        <v>0.375</v>
       </c>
       <c r="G60">
-        <v>0.04878048780487805</v>
+        <v>0.2083333333333333</v>
       </c>
     </row>
     <row r="61" spans="1:7">
@@ -2077,22 +2062,22 @@
         <v>69</v>
       </c>
       <c r="B61" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="C61">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="D61">
         <v>7</v>
       </c>
       <c r="E61">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F61">
-        <v>0.3333333333333333</v>
+        <v>0.1891891891891892</v>
       </c>
       <c r="G61">
-        <v>0.2857142857142857</v>
+        <v>0.1081081081081081</v>
       </c>
     </row>
     <row r="62" spans="1:7">
@@ -2103,19 +2088,19 @@
         <v>8</v>
       </c>
       <c r="C62">
-        <v>97</v>
+        <v>74</v>
       </c>
       <c r="D62">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="E62">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="F62">
-        <v>0.3814432989690721</v>
+        <v>0.1351351351351351</v>
       </c>
       <c r="G62">
-        <v>0.2061855670103093</v>
+        <v>0.08108108108108109</v>
       </c>
     </row>
     <row r="63" spans="1:7">
@@ -2126,19 +2111,19 @@
         <v>8</v>
       </c>
       <c r="C63">
-        <v>37</v>
+        <v>68</v>
       </c>
       <c r="D63">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="E63">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="F63">
-        <v>0.1891891891891892</v>
+        <v>0.4411764705882353</v>
       </c>
       <c r="G63">
-        <v>0.1081081081081081</v>
+        <v>0.2352941176470588</v>
       </c>
     </row>
     <row r="64" spans="1:7">
@@ -2149,19 +2134,19 @@
         <v>8</v>
       </c>
       <c r="C64">
-        <v>74</v>
+        <v>26</v>
       </c>
       <c r="D64">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E64">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F64">
-        <v>0.1351351351351351</v>
+        <v>0.03846153846153846</v>
       </c>
       <c r="G64">
-        <v>0.08108108108108109</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65" spans="1:7">
@@ -2169,22 +2154,22 @@
         <v>73</v>
       </c>
       <c r="B65" t="s">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="C65">
-        <v>68</v>
+        <v>22</v>
       </c>
       <c r="D65">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="E65">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="F65">
-        <v>0.4411764705882353</v>
+        <v>0.1363636363636364</v>
       </c>
       <c r="G65">
-        <v>0.2352941176470588</v>
+        <v>0.04545454545454546</v>
       </c>
     </row>
     <row r="66" spans="1:7">
@@ -2195,19 +2180,19 @@
         <v>8</v>
       </c>
       <c r="C66">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="D66">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="E66">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="F66">
-        <v>0.03846153846153846</v>
+        <v>0.5483870967741935</v>
       </c>
       <c r="G66">
-        <v>0</v>
+        <v>0.3870967741935484</v>
       </c>
     </row>
     <row r="67" spans="1:7">
@@ -2215,22 +2200,22 @@
         <v>75</v>
       </c>
       <c r="B67" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="C67">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D67">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="E67">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="F67">
-        <v>0.1363636363636364</v>
+        <v>0.8</v>
       </c>
       <c r="G67">
-        <v>0.04545454545454546</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="68" spans="1:7">
@@ -2241,19 +2226,19 @@
         <v>8</v>
       </c>
       <c r="C68">
-        <v>23</v>
+        <v>56</v>
       </c>
       <c r="D68">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="E68">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="F68">
-        <v>0.5652173913043478</v>
+        <v>0.4464285714285715</v>
       </c>
       <c r="G68">
-        <v>0.08695652173913043</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="69" spans="1:7">
@@ -2264,19 +2249,19 @@
         <v>8</v>
       </c>
       <c r="C69">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D69">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E69">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F69">
-        <v>0.5483870967741935</v>
+        <v>0.625</v>
       </c>
       <c r="G69">
-        <v>0.3870967741935484</v>
+        <v>0.34375</v>
       </c>
     </row>
     <row r="70" spans="1:7">
@@ -2284,22 +2269,22 @@
         <v>78</v>
       </c>
       <c r="B70" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C70">
-        <v>20</v>
+        <v>49</v>
       </c>
       <c r="D70">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E70">
         <v>11</v>
       </c>
       <c r="F70">
-        <v>0.8</v>
+        <v>0.3673469387755102</v>
       </c>
       <c r="G70">
-        <v>0.55</v>
+        <v>0.2244897959183673</v>
       </c>
     </row>
     <row r="71" spans="1:7">
@@ -2310,19 +2295,19 @@
         <v>8</v>
       </c>
       <c r="C71">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D71">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="E71">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="F71">
-        <v>0.72</v>
+        <v>0.5454545454545454</v>
       </c>
       <c r="G71">
-        <v>0.4</v>
+        <v>0.3181818181818182</v>
       </c>
     </row>
     <row r="72" spans="1:7">
@@ -2333,19 +2318,19 @@
         <v>8</v>
       </c>
       <c r="C72">
-        <v>58</v>
+        <v>31</v>
       </c>
       <c r="D72">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="E72">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="F72">
-        <v>0.4655172413793103</v>
+        <v>0.4516129032258064</v>
       </c>
       <c r="G72">
-        <v>0.2758620689655172</v>
+        <v>0.1935483870967742</v>
       </c>
     </row>
     <row r="73" spans="1:7">
@@ -2353,22 +2338,22 @@
         <v>81</v>
       </c>
       <c r="B73" t="s">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="C73">
-        <v>32</v>
+        <v>56</v>
       </c>
       <c r="D73">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="E73">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="F73">
-        <v>0.625</v>
+        <v>0.125</v>
       </c>
       <c r="G73">
-        <v>0.34375</v>
+        <v>0.08928571428571429</v>
       </c>
     </row>
     <row r="74" spans="1:7">
@@ -2376,22 +2361,22 @@
         <v>82</v>
       </c>
       <c r="B74" t="s">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="C74">
-        <v>49</v>
+        <v>69</v>
       </c>
       <c r="D74">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E74">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="F74">
-        <v>0.3673469387755102</v>
+        <v>0.2463768115942029</v>
       </c>
       <c r="G74">
-        <v>0.2244897959183673</v>
+        <v>0.2318840579710145</v>
       </c>
     </row>
     <row r="75" spans="1:7">
@@ -2399,111 +2384,111 @@
         <v>83</v>
       </c>
       <c r="B75" t="s">
-        <v>8</v>
+        <v>84</v>
       </c>
       <c r="C75">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D75">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="E75">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="F75">
-        <v>0.5454545454545454</v>
+        <v>0.15</v>
       </c>
       <c r="G75">
-        <v>0.3181818181818182</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76" spans="1:7">
       <c r="A76" t="s">
+        <v>85</v>
+      </c>
+      <c r="B76" t="s">
         <v>84</v>
-      </c>
-      <c r="B76" t="s">
-        <v>8</v>
       </c>
       <c r="C76">
         <v>31</v>
       </c>
       <c r="D76">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="E76">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F76">
-        <v>0.4516129032258064</v>
+        <v>0.06451612903225806</v>
       </c>
       <c r="G76">
-        <v>0.1935483870967742</v>
+        <v>0</v>
       </c>
     </row>
     <row r="77" spans="1:7">
       <c r="A77" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B77" t="s">
         <v>30</v>
       </c>
       <c r="C77">
-        <v>56</v>
+        <v>21</v>
       </c>
       <c r="D77">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E77">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F77">
-        <v>0.125</v>
+        <v>0.4761904761904762</v>
       </c>
       <c r="G77">
-        <v>0.08928571428571429</v>
+        <v>0.04761904761904762</v>
       </c>
     </row>
     <row r="78" spans="1:7">
       <c r="A78" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B78" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="C78">
-        <v>69</v>
+        <v>41</v>
       </c>
       <c r="D78">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="E78">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="F78">
-        <v>0.2463768115942029</v>
+        <v>0.2195121951219512</v>
       </c>
       <c r="G78">
-        <v>0.2318840579710145</v>
+        <v>0.1219512195121951</v>
       </c>
     </row>
     <row r="79" spans="1:7">
       <c r="A79" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B79" t="s">
-        <v>88</v>
+        <v>8</v>
       </c>
       <c r="C79">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="D79">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E79">
         <v>0</v>
       </c>
       <c r="F79">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="G79">
         <v>0</v>
@@ -2514,22 +2499,22 @@
         <v>89</v>
       </c>
       <c r="B80" t="s">
-        <v>88</v>
+        <v>8</v>
       </c>
       <c r="C80">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D80">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E80">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F80">
-        <v>0.06451612903225806</v>
+        <v>0.1724137931034483</v>
       </c>
       <c r="G80">
-        <v>0</v>
+        <v>0.103448275862069</v>
       </c>
     </row>
     <row r="81" spans="1:7">
@@ -2537,22 +2522,22 @@
         <v>90</v>
       </c>
       <c r="B81" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="C81">
-        <v>21</v>
+        <v>135</v>
       </c>
       <c r="D81">
-        <v>10</v>
+        <v>69</v>
       </c>
       <c r="E81">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="F81">
-        <v>0.4761904761904762</v>
+        <v>0.5111111111111111</v>
       </c>
       <c r="G81">
-        <v>0.04761904761904762</v>
+        <v>0.2074074074074074</v>
       </c>
     </row>
     <row r="82" spans="1:7">
@@ -2563,19 +2548,19 @@
         <v>8</v>
       </c>
       <c r="C82">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="D82">
         <v>9</v>
       </c>
       <c r="E82">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F82">
-        <v>0.2195121951219512</v>
+        <v>0.3461538461538461</v>
       </c>
       <c r="G82">
-        <v>0.1219512195121951</v>
+        <v>0.2307692307692308</v>
       </c>
     </row>
     <row r="83" spans="1:7">
@@ -2586,19 +2571,19 @@
         <v>8</v>
       </c>
       <c r="C83">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="D83">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E83">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F83">
-        <v>0</v>
+        <v>0.1428571428571428</v>
       </c>
       <c r="G83">
-        <v>0</v>
+        <v>0.04761904761904762</v>
       </c>
     </row>
     <row r="84" spans="1:7">
@@ -2609,19 +2594,19 @@
         <v>8</v>
       </c>
       <c r="C84">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="D84">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="E84">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="F84">
-        <v>0.1724137931034483</v>
+        <v>0.3061224489795918</v>
       </c>
       <c r="G84">
-        <v>0.103448275862069</v>
+        <v>0.1836734693877551</v>
       </c>
     </row>
     <row r="85" spans="1:7">
@@ -2632,19 +2617,19 @@
         <v>8</v>
       </c>
       <c r="C85">
-        <v>140</v>
+        <v>47</v>
       </c>
       <c r="D85">
-        <v>74</v>
+        <v>12</v>
       </c>
       <c r="E85">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="F85">
-        <v>0.5285714285714286</v>
+        <v>0.2553191489361702</v>
       </c>
       <c r="G85">
-        <v>0.2071428571428572</v>
+        <v>0</v>
       </c>
     </row>
     <row r="86" spans="1:7">
@@ -2652,22 +2637,22 @@
         <v>95</v>
       </c>
       <c r="B86" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="C86">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D86">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E86">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="F86">
-        <v>0.3461538461538461</v>
+        <v>0.25</v>
       </c>
       <c r="G86">
-        <v>0.2307692307692308</v>
+        <v>0.04166666666666666</v>
       </c>
     </row>
     <row r="87" spans="1:7">
@@ -2675,22 +2660,22 @@
         <v>96</v>
       </c>
       <c r="B87" t="s">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="C87">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="D87">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E87">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F87">
-        <v>0.1428571428571428</v>
+        <v>0.225</v>
       </c>
       <c r="G87">
-        <v>0.04761904761904762</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="88" spans="1:7">
@@ -2701,19 +2686,19 @@
         <v>8</v>
       </c>
       <c r="C88">
-        <v>49</v>
+        <v>95</v>
       </c>
       <c r="D88">
+        <v>27</v>
+      </c>
+      <c r="E88">
         <v>15</v>
       </c>
-      <c r="E88">
-        <v>9</v>
-      </c>
       <c r="F88">
-        <v>0.3061224489795918</v>
+        <v>0.2842105263157895</v>
       </c>
       <c r="G88">
-        <v>0.1836734693877551</v>
+        <v>0.1578947368421053</v>
       </c>
     </row>
     <row r="89" spans="1:7">
@@ -2724,19 +2709,19 @@
         <v>8</v>
       </c>
       <c r="C89">
-        <v>47</v>
+        <v>29</v>
       </c>
       <c r="D89">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E89">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F89">
-        <v>0.2553191489361702</v>
+        <v>0.1724137931034483</v>
       </c>
       <c r="G89">
-        <v>0</v>
+        <v>0.03448275862068965</v>
       </c>
     </row>
     <row r="90" spans="1:7">
@@ -2744,22 +2729,22 @@
         <v>99</v>
       </c>
       <c r="B90" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="C90">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D90">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E90">
         <v>1</v>
       </c>
       <c r="F90">
-        <v>0.25</v>
+        <v>0.1</v>
       </c>
       <c r="G90">
-        <v>0.04166666666666666</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="91" spans="1:7">
@@ -2767,22 +2752,22 @@
         <v>100</v>
       </c>
       <c r="B91" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="C91">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="D91">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E91">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F91">
-        <v>0.225</v>
+        <v>0.09677419354838709</v>
       </c>
       <c r="G91">
-        <v>0.125</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92" spans="1:7">
@@ -2790,22 +2775,22 @@
         <v>101</v>
       </c>
       <c r="B92" t="s">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="C92">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D92">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="E92">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="F92">
-        <v>0.2842105263157895</v>
+        <v>0.1382978723404255</v>
       </c>
       <c r="G92">
-        <v>0.1578947368421053</v>
+        <v>0.02127659574468085</v>
       </c>
     </row>
     <row r="93" spans="1:7">
@@ -2813,10 +2798,10 @@
         <v>102</v>
       </c>
       <c r="B93" t="s">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="C93">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="D93">
         <v>5</v>
@@ -2825,10 +2810,10 @@
         <v>1</v>
       </c>
       <c r="F93">
-        <v>0.1724137931034483</v>
+        <v>0.08771929824561403</v>
       </c>
       <c r="G93">
-        <v>0.03448275862068965</v>
+        <v>0.01754385964912281</v>
       </c>
     </row>
     <row r="94" spans="1:7">
@@ -2839,19 +2824,19 @@
         <v>8</v>
       </c>
       <c r="C94">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D94">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="E94">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F94">
-        <v>0.1</v>
+        <v>0.5217391304347826</v>
       </c>
       <c r="G94">
-        <v>0.05</v>
+        <v>0.3478260869565217</v>
       </c>
     </row>
     <row r="95" spans="1:7">
@@ -2862,19 +2847,19 @@
         <v>8</v>
       </c>
       <c r="C95">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="D95">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="E95">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F95">
-        <v>0.09677419354838709</v>
+        <v>0.475</v>
       </c>
       <c r="G95">
-        <v>0</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="96" spans="1:7">
@@ -2882,137 +2867,22 @@
         <v>105</v>
       </c>
       <c r="B96" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="C96">
-        <v>94</v>
+        <v>39</v>
       </c>
       <c r="D96">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E96">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F96">
-        <v>0.1382978723404255</v>
+        <v>0.4358974358974359</v>
       </c>
       <c r="G96">
-        <v>0.02127659574468085</v>
-      </c>
-    </row>
-    <row r="97" spans="1:7">
-      <c r="A97" t="s">
-        <v>106</v>
-      </c>
-      <c r="B97" t="s">
-        <v>30</v>
-      </c>
-      <c r="C97">
-        <v>57</v>
-      </c>
-      <c r="D97">
-        <v>5</v>
-      </c>
-      <c r="E97">
-        <v>1</v>
-      </c>
-      <c r="F97">
-        <v>0.08771929824561403</v>
-      </c>
-      <c r="G97">
-        <v>0.01754385964912281</v>
-      </c>
-    </row>
-    <row r="98" spans="1:7">
-      <c r="A98" t="s">
-        <v>107</v>
-      </c>
-      <c r="B98" t="s">
-        <v>8</v>
-      </c>
-      <c r="C98">
-        <v>23</v>
-      </c>
-      <c r="D98">
-        <v>12</v>
-      </c>
-      <c r="E98">
-        <v>8</v>
-      </c>
-      <c r="F98">
-        <v>0.5217391304347826</v>
-      </c>
-      <c r="G98">
-        <v>0.3478260869565217</v>
-      </c>
-    </row>
-    <row r="99" spans="1:7">
-      <c r="A99" t="s">
-        <v>108</v>
-      </c>
-      <c r="B99" t="s">
-        <v>8</v>
-      </c>
-      <c r="C99">
-        <v>40</v>
-      </c>
-      <c r="D99">
-        <v>19</v>
-      </c>
-      <c r="E99">
-        <v>10</v>
-      </c>
-      <c r="F99">
-        <v>0.475</v>
-      </c>
-      <c r="G99">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="100" spans="1:7">
-      <c r="A100" t="s">
-        <v>109</v>
-      </c>
-      <c r="B100" t="s">
-        <v>8</v>
-      </c>
-      <c r="C100">
-        <v>31</v>
-      </c>
-      <c r="D100">
-        <v>31</v>
-      </c>
-      <c r="E100">
-        <v>3</v>
-      </c>
-      <c r="F100">
-        <v>1</v>
-      </c>
-      <c r="G100">
-        <v>0.09677419354838709</v>
-      </c>
-    </row>
-    <row r="101" spans="1:7">
-      <c r="A101" t="s">
-        <v>110</v>
-      </c>
-      <c r="B101" t="s">
-        <v>8</v>
-      </c>
-      <c r="C101">
-        <v>40</v>
-      </c>
-      <c r="D101">
-        <v>18</v>
-      </c>
-      <c r="E101">
-        <v>10</v>
-      </c>
-      <c r="F101">
-        <v>0.45</v>
-      </c>
-      <c r="G101">
-        <v>0.25</v>
+        <v>0.2564102564102564</v>
       </c>
     </row>
   </sheetData>

</xml_diff>